<commit_message>
News section, sold-regions stat, auto-rotating maps, world map pulse
- News sheet in kittens.xlsx renders 猫舍动态 timeline (出生/出售/公告 tags)
- 售往地区 chips computed from sold kittens' 新家地址
- Map pane auto-rotates world/China every 5.5s (click stops auto)
- World map now has Chengdu pulse marker

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="小猫数据" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="种猫" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新闻" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1137,7 +1138,7 @@
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1161,7 +1162,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1185,7 +1186,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1700,7 +1701,60 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>公告</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Shakoshako 猫舍官网全新上线，欢迎关注！</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1840,6 +1894,16 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>「新闻」工作表：日期(2026-08-05格式)、类型(出生/出售/公告)、内容。网站 News 区按日期倒序显示，最多显示 8 条。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Kitten footprints map in hero, names for sold kittens, feedback section, collapsible news before kittens, about moved up with live stats
- 名字/家长反馈/设置 added to kittens.xlsx (驺驺 → 荷兰 recorded)
- Hero shows 🐾 小猫足迹 world map with destination dots
- About section relocated before kittens with auto counts (在售/已售)
- News section relocated before kittens, collapsible header
- Sold cards show custom name with color/sex subtitle and new home

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -10,7 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="小猫数据" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="种猫" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新闻" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="家长反馈" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设置" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -452,6 +454,7 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -495,6 +498,11 @@
           <t>妈妈</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>名字</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1186,7 +1194,16 @@
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="n"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>驺驺</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1754,7 +1771,81 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>小猫名字</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>值</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>成立日期</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1904,6 +1995,37 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>小猫表新增「名字」列：填写后卡片标题显示名字（花色性别变为小字副标题）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>「家长反馈」工作表：日期、小猫名字、内容。填写后网站显示家长反馈区。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>新家地址可填国内城市或国家（如 北京、荷兰），首页的售往地图会自动打点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>「设置」工作表：成立日期填如 2022 或 2022-06，填写后显示在关于我们的统计里。在售/已售数量自动统计。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record Aug 2 sales (银虎斑弟弟→黑龙江, 烟灰色弟弟→重庆); province geo; feedback image slots
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -606,7 +606,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -614,7 +614,11 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>重庆</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -746,7 +750,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -754,7 +758,11 @@
           <t>2025-11-05</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>黑龙江</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1718,7 +1726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1757,6 +1765,40 @@
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Shakoshako 猫舍官网全新上线，欢迎关注！</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>出售</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>银虎斑弟弟到达黑龙江的新家，开启新生活！</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>出售</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>烟灰色弟弟到达重庆的新家，开启新生活！</t>
         </is>
       </c>
     </row>
@@ -1771,12 +1813,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1793,6 +1836,11 @@
       <c r="C1" s="1" t="inlineStr">
         <is>
           <t>内容</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>图片路径</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2026,6 +2074,13 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>家长反馈的「图片路径」可选：填 assets/文件名.jpg（多张用逗号分隔），卡片会显示图片，点击可放大。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
News compact with map background, date grouping, 已定新家 wording; about first, default filter available, go-home kit block
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -1781,7 +1781,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>银虎斑弟弟到达黑龙江的新家，开启新生活！</t>
+          <t>银虎斑弟弟已定新家 · 黑龙江</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>烟灰色弟弟到达重庆的新家，开启新生活！</t>
+          <t>烟灰色弟弟已定新家 · 重庆</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1881,6 +1881,18 @@
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>新家礼包</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>幼猫粮、熟悉气味的小毯子、玩具、疫苗本与驱虫记录、电子合同、终身饲养指导</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1893,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2081,6 +2093,13 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>「设置」表新增 新家礼包：用顿号或逗号分隔物品清单，显示在购买流程下方。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Proportional about montage, 3x2 fact grid, statement as page finale, Zouzou's parents (阿泽 × 小辫子) recorded
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -1207,6 +1207,16 @@
           <t>荷兰</t>
         </is>
       </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>阿泽</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>小辫子</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>驺驺</t>

</xml_diff>

<commit_message>
Correct: 驺驺 is the blue tabby girl (5mo), moved name/home/parents
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -1154,7 +1154,26 @@
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n"/>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>阿泽</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>小辫子</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>驺驺</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1202,26 +1221,9 @@
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>荷兰</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>阿泽</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>小辫子</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>驺驺</t>
-        </is>
-      </c>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Revert guessed Aug-2 sales entries; move to TODO for cattery to fill
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -606,7 +606,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -614,11 +614,7 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>重庆</t>
-        </is>
-      </c>
+      <c r="F5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -750,7 +746,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -758,11 +754,7 @@
           <t>2025-11-05</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>黑龙江</t>
-        </is>
-      </c>
+      <c r="F10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1738,7 +1730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1777,40 +1769,6 @@
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Shakoshako 猫舍官网全新上线，欢迎关注！</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>出售</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>银虎斑弟弟已定新家 · 黑龙江</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>出售</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>烟灰色弟弟已定新家 · 重庆</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Parent side-drawer, WeChat copy-to-clipboard, world visitor dots, unified 1180px containers, night alternation (kittens light), merged statement+footer, cattery copyright, XHS icon, name format 花色·名字, intro text & photo white-edge fixes
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -1825,7 +1825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1861,6 +1861,18 @@
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>日常用品、猫粮、常用药品</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>访客地区</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>中国、荷兰</t>
         </is>
       </c>
     </row>
@@ -1875,7 +1887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2070,6 +2082,13 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>「设置」表 访客地区：顿号分隔的国家/地区清单（可从访问统计明细页查看后更新），全球地图上会自动点亮这些位置。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Strict night alternation (values light, cattery dark), sold cards hide age, montage exact alignment, first family-feedback entry (驺驺)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -1783,7 +1783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1813,6 +1813,24 @@
           <t>图片路径</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>驺驺</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>在荷兰的新家适应得很好，活泼又粘人。</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Kitten detail drawer: photo slider + parents + inline family feedback; multi-photo kitten paths; unified visitor dots on both maps; Zouzou feedback photo; process intro single line
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -1830,7 +1830,11 @@
           <t>在荷兰的新家适应得很好，活泼又粘人。</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>assets/feedback/zouzou-1.jpg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Reserved status (驺驺), FAQ accordion from Excel, WeChat/OG share card
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -11,8 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="种猫" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新闻" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="家长反馈" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设置" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="常见问题" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设置" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1138,7 +1139,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>预定</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1847,54 +1848,94 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>项目</t>
+          <t>问题</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>值</t>
+          <t>答案</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>成立日期</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr"/>
+          <t>外地/海外可以购买吗？怎么接猫？</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>可以。您可以到成都自提，也可以由我们安排航空托运；海外接猫请提前微信沟通，我们会说明流程与费用。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>新家礼包</t>
+          <t>如何预订心仪的小猫？</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>日常用品、猫粮、常用药品</t>
+          <t>通过微信沟通确认小猫后，支付 30% 定金并签订电子合同即完成预订；接猫前一天付清尾款。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>访客地区</t>
+          <t>小猫接回家时会附带什么？</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>中国、荷兰</t>
+          <t>新家礼包会随小猫一同快递寄出，内含日常用品、猫粮和常用药品；同时提供疫苗与驱虫记录。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>猫舍做了哪些健康保障？</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>种猫均进行 HCM（肥厚型心肌病）与 PKD（多囊肾）基因检测，幼猫按月龄完成疫苗和驱虫，并提供终身饲养指导。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>小猫多大可以接回家？</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>一般满 3 个月、完成基础疫苗后交付，具体以每只小猫的状态为准。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>还有其他问题？</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>欢迎通过页面下方的微信或电话直接咨询我们。</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1950,69 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>值</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>成立日期</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>新家礼包</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>日常用品、猫粮、常用药品</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>访客地区</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>中国、荷兰</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2111,6 +2214,23 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>「常见问题」工作表：问题/答案，显示在购买流程下方（可折叠）。当前答案为草拟，请核对修改。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>「是否出售」现在支持三种：否 = 待出售；预定 = 已交定金待接走（金色角标）；是 = 已出售。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
FAQ standalone color block with re-alternated tail; 已预定 wording; drop overseas FAQ entry
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -1848,7 +1848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1870,70 +1870,58 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>外地/海外可以购买吗？怎么接猫？</t>
+          <t>如何预订心仪的小猫？</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>可以。您可以到成都自提，也可以由我们安排航空托运；海外接猫请提前微信沟通，我们会说明流程与费用。</t>
+          <t>通过微信沟通确认小猫后，支付 30% 定金并签订电子合同即完成预订；接猫前一天付清尾款。</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>如何预订心仪的小猫？</t>
+          <t>小猫接回家时会附带什么？</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>通过微信沟通确认小猫后，支付 30% 定金并签订电子合同即完成预订；接猫前一天付清尾款。</t>
+          <t>新家礼包会随小猫一同快递寄出，内含日常用品、猫粮和常用药品；同时提供疫苗与驱虫记录。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>小猫接回家时会附带什么？</t>
+          <t>猫舍做了哪些健康保障？</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>新家礼包会随小猫一同快递寄出，内含日常用品、猫粮和常用药品；同时提供疫苗与驱虫记录。</t>
+          <t>种猫均进行 HCM（肥厚型心肌病）与 PKD（多囊肾）基因检测，幼猫按月龄完成疫苗和驱虫，并提供终身饲养指导。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>猫舍做了哪些健康保障？</t>
+          <t>小猫多大可以接回家？</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>种猫均进行 HCM（肥厚型心肌病）与 PKD（多囊肾）基因检测，幼猫按月龄完成疫苗和驱虫，并提供终身饲养指导。</t>
+          <t>一般满 3 个月、完成基础疫苗后交付，具体以每只小猫的状态为准。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>小猫多大可以接回家？</t>
+          <t>还有其他问题？</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>一般满 3 个月、完成基础疫苗后交付，具体以每只小猫的状态为准。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>还有其他问题？</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>欢迎通过页面下方的微信或电话直接咨询我们。</t>
         </is>

</xml_diff>